<commit_message>
Desired voltage set to 0.2V increments
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a4fd901eb976e385/Desktop/Power Supply/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="257" documentId="11_F25DC773A252ABDACC10487EC95C72D65BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2E9791B-FEE3-4B91-83EE-DE9A76C9DD7A}"/>
+  <xr:revisionPtr revIDLastSave="312" documentId="11_F25DC773A252ABDACC10487EC95C72D65BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D7B9A20-F710-4A87-83C5-E5889970BA37}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
+    <sheet name="ADC" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="17">
   <si>
     <t>Vsense</t>
   </si>
@@ -69,6 +70,24 @@
   </si>
   <si>
     <t>Go into graph filters to bring back 256 tap</t>
+  </si>
+  <si>
+    <t>Avg. Error</t>
+  </si>
+  <si>
+    <t>Ratio</t>
+  </si>
+  <si>
+    <t>R4</t>
+  </si>
+  <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>ADC</t>
+  </si>
+  <si>
+    <t>Voltage</t>
   </si>
 </sst>
 </file>
@@ -179,10 +198,10 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1446,7 +1465,40 @@
             </c:spPr>
             <c:trendlineType val="linear"/>
             <c:dispRSqr val="0"/>
-            <c:dispEq val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="0.23557340832539186"/>
+                  <c:y val="5.7252578648917122E-3"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:sysClr val="windowText" lastClr="000000"/>
+                      </a:solidFill>
+                      <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
           </c:trendline>
           <c:xVal>
             <c:numRef>
@@ -2195,6 +2247,622 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-AU"/>
+              <a:t>Analog Ratio</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Analog</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="0.20439501937150753"/>
+                  <c:y val="-2.92860588676375E-3"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:sysClr val="windowText" lastClr="000000"/>
+                      </a:solidFill>
+                      <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Data!$H$4:$H$24</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.2000000000000002</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.6</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.4</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3.6</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>3.8</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>4.2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>4.4000000000000004</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>4.5999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>4.8</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>5.2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>5.4</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>5.6</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>5.8</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Data!$J$4:$J$24</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>146</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>164</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>177</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>192</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>206</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>219</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>232</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>247</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>258</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>271</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>287</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>305</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>316</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>329</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>343</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>358</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>375</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>376</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>395</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>416</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000007-8C23-47CA-8CBB-AB3486FD02AB}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1677198032"/>
+        <c:axId val="1677198512"/>
+        <c:extLst/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1677198032"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="6"/>
+          <c:min val="2"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-AU"/>
+                  <a:t>Input Voltage (V)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1677198512"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1677198512"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-AU"/>
+                  <a:t>Target</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-AU" baseline="0"/>
+                  <a:t> Error (V)</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-AU"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-AU"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1677198032"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr b="0">
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+          <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+          <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -2275,6 +2943,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -2792,6 +3500,522 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -3378,6 +4602,44 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>29307</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>381958</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>161542</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{83D729AB-7FB1-46AD-B96F-DDE88090D8D9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3649,7 +4911,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:S51"/>
+  <dimension ref="B2:S55"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -3659,12 +4921,12 @@
     <col min="5" max="5" width="6.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25.5703125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="6.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="6.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.140625" style="1"/>
+    <col min="13" max="13" width="28.7109375" style="1" customWidth="1"/>
     <col min="14" max="14" width="6.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -3674,27 +4936,27 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:18" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="H2" s="8" t="s">
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="H2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="N2" s="8" t="s">
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="N2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="O2" s="8"/>
-      <c r="P2" s="8"/>
-      <c r="Q2" s="8"/>
-      <c r="R2" s="8"/>
+      <c r="O2" s="9"/>
+      <c r="P2" s="9"/>
+      <c r="Q2" s="9"/>
+      <c r="R2" s="9"/>
     </row>
     <row r="3" spans="2:18" ht="15.75" x14ac:dyDescent="0.2">
       <c r="B3" s="4" t="s">
@@ -4674,7 +5936,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
       <c r="B23" s="2">
         <v>5.8</v>
       </c>
@@ -4692,6 +5954,9 @@
         <f t="shared" si="1"/>
         <v>67.684021543985637</v>
       </c>
+      <c r="G23" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="H23" s="2">
         <v>5.8</v>
       </c>
@@ -4708,6 +5973,9 @@
       <c r="L23" s="6">
         <f t="shared" si="3"/>
         <v>67.406143344709889</v>
+      </c>
+      <c r="M23" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="N23" s="2">
         <v>5.8</v>
@@ -4741,6 +6009,10 @@
         <f t="shared" si="1"/>
         <v>67.637540453074436</v>
       </c>
+      <c r="G24" s="2">
+        <f>AVERAGE(E4:E24)</f>
+        <v>-0.43571428571428583</v>
+      </c>
       <c r="H24" s="2">
         <v>6</v>
       </c>
@@ -4757,6 +6029,10 @@
       <c r="L24" s="6">
         <f t="shared" si="3"/>
         <v>67.313915857605181</v>
+      </c>
+      <c r="M24" s="2">
+        <f>AVERAGE(K4:K24)</f>
+        <v>-8.1904761904761939E-2</v>
       </c>
       <c r="N24" s="2">
         <v>6</v>
@@ -4773,7 +6049,7 @@
       </c>
     </row>
     <row r="31" spans="2:19" x14ac:dyDescent="0.2">
-      <c r="S31" s="9" t="s">
+      <c r="S31" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -4801,6 +6077,31 @@
       <c r="I51" s="6">
         <f>200/3</f>
         <v>66.666666666666671</v>
+      </c>
+    </row>
+    <row r="53" spans="8:9" ht="15" x14ac:dyDescent="0.2">
+      <c r="H53" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I53" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="54" spans="8:9" x14ac:dyDescent="0.2">
+      <c r="H54" s="6">
+        <v>7970</v>
+      </c>
+      <c r="I54" s="6">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="55" spans="8:9" ht="15" x14ac:dyDescent="0.2">
+      <c r="H55" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="I55" s="2">
+        <f>I54/H54</f>
+        <v>1.5056461731493098</v>
       </c>
     </row>
   </sheetData>
@@ -4813,4 +6114,150 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C187DCCE-8E32-44A3-9556-14C14F1C388A}">
+  <dimension ref="B3:C24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="3" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B4" s="2">
+        <v>0.72499999999999998</v>
+      </c>
+      <c r="C4" s="2">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B5" s="2"/>
+      <c r="C5" s="2">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B6" s="2"/>
+      <c r="C6" s="2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B7" s="2"/>
+      <c r="C7" s="2">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B8" s="2"/>
+      <c r="C8" s="2">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B9" s="2"/>
+      <c r="C9" s="2">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B10" s="2"/>
+      <c r="C10" s="2">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B11" s="2"/>
+      <c r="C11" s="2">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B12" s="2"/>
+      <c r="C12" s="2">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B13" s="2"/>
+      <c r="C13" s="2">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B14" s="2"/>
+      <c r="C14" s="2">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B15" s="2"/>
+      <c r="C15" s="2">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B16" s="2"/>
+      <c r="C16" s="2">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B17" s="2"/>
+      <c r="C17" s="2">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18" s="2"/>
+      <c r="C18" s="2">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="2"/>
+      <c r="C19" s="2">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B20" s="2"/>
+      <c r="C20" s="2">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B21" s="2"/>
+      <c r="C21" s="2">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B22" s="2"/>
+      <c r="C22" s="2">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B23" s="2"/>
+      <c r="C23" s="2">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B24" s="2"/>
+      <c r="C24" s="2">
+        <v>416</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Data gathered and Vsense offset added. Vsense is very close to Vout
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a4fd901eb976e385/Desktop/Power Supply/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="312" documentId="11_F25DC773A252ABDACC10487EC95C72D65BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D7B9A20-F710-4A87-83C5-E5889970BA37}"/>
+  <xr:revisionPtr revIDLastSave="406" documentId="11_F25DC773A252ABDACC10487EC95C72D65BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D58204A0-B3F4-4E5E-ADDA-C6F9C32CB9FD}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
-    <sheet name="ADC" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,15 +36,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
   <si>
     <t>Vsense</t>
   </si>
   <si>
     <t>No Feedback (Calculate Resistance)</t>
-  </si>
-  <si>
-    <t>Feedback System (128 Tap)</t>
   </si>
   <si>
     <t>X</t>
@@ -58,9 +54,6 @@
   </si>
   <si>
     <t>Output</t>
-  </si>
-  <si>
-    <t>Feedback System (256 Tap)</t>
   </si>
   <si>
     <t>Analog</t>
@@ -84,10 +77,22 @@
     <t>R3</t>
   </si>
   <si>
-    <t>ADC</t>
+    <t>Feedback System v1 (128 Tap)</t>
   </si>
   <si>
-    <t>Voltage</t>
+    <t>Vsense (V)</t>
+  </si>
+  <si>
+    <t>I/O Error</t>
+  </si>
+  <si>
+    <t>Vsense Error</t>
+  </si>
+  <si>
+    <t>Avg. Vsense Error</t>
+  </si>
+  <si>
+    <t>Feedback System v2 (256 Tap) (0.1V accuracy)</t>
   </si>
 </sst>
 </file>
@@ -646,6 +651,170 @@
             </c:ext>
           </c:extLst>
         </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Data!$N$6:$N$24</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>2.4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.6</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3.2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3.4</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4.2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>4.4000000000000004</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>4.5999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>4.8</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>5.2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>5.4</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>5.6</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>5.8</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Data!$Q$6:$Q$24</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>-0.14999999999999991</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5.0000000000000266E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4.0000000000000036E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6.0000000000000053E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.0000000000000036E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.0000000000000036E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4.0000000000000036E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4.0000000000000036E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>6.0000000000000053E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-9.9999999999997868E-3</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-2.0000000000000462E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>9.9999999999997868E-3</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>1.9999999999999574E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-9.9999999999997868E-3</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-4.9999999999999822E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>1.9999999999999574E-2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-7.0000000000000284E-2</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-1.9999999999999574E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-63E1-4D82-B0CC-A5A8E5FDCE7E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
@@ -656,203 +825,7 @@
         </c:dLbls>
         <c:axId val="1677198032"/>
         <c:axId val="1677198512"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="2"/>
-                <c:order val="2"/>
-                <c:tx>
-                  <c:v>Feedback (256 Tap)</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="25400" cap="rnd">
-                    <a:noFill/>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="circle"/>
-                  <c:size val="5"/>
-                  <c:spPr>
-                    <a:solidFill>
-                      <a:schemeClr val="accent3"/>
-                    </a:solidFill>
-                    <a:ln w="9525">
-                      <a:solidFill>
-                        <a:schemeClr val="accent3"/>
-                      </a:solidFill>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Data!$N$4:$N$24</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="21"/>
-                      <c:pt idx="0">
-                        <c:v>2</c:v>
-                      </c:pt>
-                      <c:pt idx="1">
-                        <c:v>2.2000000000000002</c:v>
-                      </c:pt>
-                      <c:pt idx="2">
-                        <c:v>2.4</c:v>
-                      </c:pt>
-                      <c:pt idx="3">
-                        <c:v>2.6</c:v>
-                      </c:pt>
-                      <c:pt idx="4">
-                        <c:v>2.8</c:v>
-                      </c:pt>
-                      <c:pt idx="5">
-                        <c:v>3</c:v>
-                      </c:pt>
-                      <c:pt idx="6">
-                        <c:v>3.2</c:v>
-                      </c:pt>
-                      <c:pt idx="7">
-                        <c:v>3.4</c:v>
-                      </c:pt>
-                      <c:pt idx="8">
-                        <c:v>3.6</c:v>
-                      </c:pt>
-                      <c:pt idx="9">
-                        <c:v>3.8</c:v>
-                      </c:pt>
-                      <c:pt idx="10">
-                        <c:v>4</c:v>
-                      </c:pt>
-                      <c:pt idx="11">
-                        <c:v>4.2</c:v>
-                      </c:pt>
-                      <c:pt idx="12">
-                        <c:v>4.4000000000000004</c:v>
-                      </c:pt>
-                      <c:pt idx="13">
-                        <c:v>4.5999999999999996</c:v>
-                      </c:pt>
-                      <c:pt idx="14">
-                        <c:v>4.8</c:v>
-                      </c:pt>
-                      <c:pt idx="15">
-                        <c:v>5</c:v>
-                      </c:pt>
-                      <c:pt idx="16">
-                        <c:v>5.2</c:v>
-                      </c:pt>
-                      <c:pt idx="17">
-                        <c:v>5.4</c:v>
-                      </c:pt>
-                      <c:pt idx="18">
-                        <c:v>5.6</c:v>
-                      </c:pt>
-                      <c:pt idx="19">
-                        <c:v>5.8</c:v>
-                      </c:pt>
-                      <c:pt idx="20">
-                        <c:v>6</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Data!$Q$4:$Q$24</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="21"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="1">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="2">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="3">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="4">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="5">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="6">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="7">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="8">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="9">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="10">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="11">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="12">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="13">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="14">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="15">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="16">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="17">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="18">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="19">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="20">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000000-63E1-4D82-B0CC-A5A8E5FDCE7E}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-          </c:ext>
-        </c:extLst>
+        <c:extLst/>
       </c:scatterChart>
       <c:valAx>
         <c:axId val="1677198032"/>
@@ -1429,7 +1402,7 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>Feedback</c:v>
+            <c:v>Feedback 128</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="25400" cap="rnd">
@@ -1465,40 +1438,7 @@
             </c:spPr>
             <c:trendlineType val="linear"/>
             <c:dispRSqr val="0"/>
-            <c:dispEq val="1"/>
-            <c:trendlineLbl>
-              <c:layout>
-                <c:manualLayout>
-                  <c:x val="0.23557340832539186"/>
-                  <c:y val="5.7252578648917122E-3"/>
-                </c:manualLayout>
-              </c:layout>
-              <c:numFmt formatCode="General" sourceLinked="0"/>
-              <c:spPr>
-                <a:noFill/>
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-              <c:txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr>
-                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                      <a:solidFill>
-                        <a:sysClr val="windowText" lastClr="000000"/>
-                      </a:solidFill>
-                      <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-                      <a:ea typeface="+mn-ea"/>
-                      <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-                    </a:defRPr>
-                  </a:pPr>
-                  <a:endParaRPr lang="en-US"/>
-                </a:p>
-              </c:txPr>
-            </c:trendlineLbl>
+            <c:dispEq val="0"/>
           </c:trendline>
           <c:xVal>
             <c:numRef>
@@ -1648,6 +1588,187 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-B3F4-4908-8561-D46CB255E536}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>Feedback 256</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent4"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Data!$N$6:$N$24</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>2.4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.6</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3.2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3.4</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4.2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>4.4000000000000004</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>4.5999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>4.8</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>5.2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>5.4</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>5.6</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>5.8</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Data!$R$6:$R$24</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>66.595294117647072</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>67.130196078431368</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>67.458695652173915</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>67.27210884353741</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>67.336708860759501</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>67.185119047619054</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>67.050561797752806</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>67.474468085106395</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>67.507614213197968</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>67.390023752969128</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>67.27</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>67.314285714285703</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>67.630480167014611</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>67.652208835341369</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>67.545489443378131</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>67.699449541284395</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>67.588888888888889</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>67.502896081771709</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>67.633554817275751</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-FF1C-4292-98D3-5F46D73CA5ED}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1740,203 +1861,7 @@
         </c:dLbls>
         <c:axId val="1677198032"/>
         <c:axId val="1677198512"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="3"/>
-                <c:order val="2"/>
-                <c:tx>
-                  <c:v>Feedback (256 Tap)</c:v>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="25400" cap="rnd">
-                    <a:noFill/>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="circle"/>
-                  <c:size val="5"/>
-                  <c:spPr>
-                    <a:solidFill>
-                      <a:schemeClr val="accent4"/>
-                    </a:solidFill>
-                    <a:ln w="9525">
-                      <a:solidFill>
-                        <a:schemeClr val="accent4"/>
-                      </a:solidFill>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Data!$N$4:$N$24</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="21"/>
-                      <c:pt idx="0">
-                        <c:v>2</c:v>
-                      </c:pt>
-                      <c:pt idx="1">
-                        <c:v>2.2000000000000002</c:v>
-                      </c:pt>
-                      <c:pt idx="2">
-                        <c:v>2.4</c:v>
-                      </c:pt>
-                      <c:pt idx="3">
-                        <c:v>2.6</c:v>
-                      </c:pt>
-                      <c:pt idx="4">
-                        <c:v>2.8</c:v>
-                      </c:pt>
-                      <c:pt idx="5">
-                        <c:v>3</c:v>
-                      </c:pt>
-                      <c:pt idx="6">
-                        <c:v>3.2</c:v>
-                      </c:pt>
-                      <c:pt idx="7">
-                        <c:v>3.4</c:v>
-                      </c:pt>
-                      <c:pt idx="8">
-                        <c:v>3.6</c:v>
-                      </c:pt>
-                      <c:pt idx="9">
-                        <c:v>3.8</c:v>
-                      </c:pt>
-                      <c:pt idx="10">
-                        <c:v>4</c:v>
-                      </c:pt>
-                      <c:pt idx="11">
-                        <c:v>4.2</c:v>
-                      </c:pt>
-                      <c:pt idx="12">
-                        <c:v>4.4000000000000004</c:v>
-                      </c:pt>
-                      <c:pt idx="13">
-                        <c:v>4.5999999999999996</c:v>
-                      </c:pt>
-                      <c:pt idx="14">
-                        <c:v>4.8</c:v>
-                      </c:pt>
-                      <c:pt idx="15">
-                        <c:v>5</c:v>
-                      </c:pt>
-                      <c:pt idx="16">
-                        <c:v>5.2</c:v>
-                      </c:pt>
-                      <c:pt idx="17">
-                        <c:v>5.4</c:v>
-                      </c:pt>
-                      <c:pt idx="18">
-                        <c:v>5.6</c:v>
-                      </c:pt>
-                      <c:pt idx="19">
-                        <c:v>5.8</c:v>
-                      </c:pt>
-                      <c:pt idx="20">
-                        <c:v>6</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Data!$R$4:$R$24</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>0.00</c:formatCode>
-                      <c:ptCount val="21"/>
-                      <c:pt idx="0">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="1">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="2">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="3">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="4">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="5">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="6">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="7">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="8">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="9">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="10">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="11">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="12">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="13">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="14">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="15">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="16">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="17">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="18">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="19">
-                        <c:v>0</c:v>
-                      </c:pt>
-                      <c:pt idx="20">
-                        <c:v>0</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000003-FF1C-4292-98D3-5F46D73CA5ED}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-          </c:ext>
-        </c:extLst>
+        <c:extLst/>
       </c:scatterChart>
       <c:valAx>
         <c:axId val="1677198032"/>
@@ -2279,7 +2204,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-AU"/>
-              <a:t>Analog Ratio</a:t>
+              <a:t>Output vs Vsense</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -2319,9 +2244,6 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:tx>
-            <c:v>Analog</c:v>
-          </c:tx>
           <c:spPr>
             <a:ln w="25400" cap="rnd">
               <a:noFill/>
@@ -2393,144 +2315,132 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Data!$H$4:$H$24</c:f>
+              <c:f>Data!$O$6:$O$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="21"/>
+                <c:ptCount val="19"/>
                 <c:pt idx="0">
-                  <c:v>2</c:v>
+                  <c:v>2.5499999999999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.2000000000000002</c:v>
+                  <c:v>2.5499999999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.4</c:v>
+                  <c:v>2.76</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2.6</c:v>
+                  <c:v>2.94</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2.8</c:v>
+                  <c:v>3.16</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3</c:v>
+                  <c:v>3.36</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3.2</c:v>
+                  <c:v>3.56</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>3.4</c:v>
+                  <c:v>3.76</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3.6</c:v>
+                  <c:v>3.94</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3.8</c:v>
+                  <c:v>4.21</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>4</c:v>
+                  <c:v>4.4000000000000004</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>4.2</c:v>
+                  <c:v>4.62</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>4.4000000000000004</c:v>
+                  <c:v>4.79</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>4.5999999999999996</c:v>
+                  <c:v>4.9800000000000004</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>4.8</c:v>
+                  <c:v>5.21</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>5</c:v>
+                  <c:v>5.45</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>5.2</c:v>
+                  <c:v>5.58</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>5.4</c:v>
+                  <c:v>5.87</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>5.6</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>5.8</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>6</c:v>
+                  <c:v>6.02</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Data!$J$4:$J$24</c:f>
+              <c:f>Data!$S$6:$S$24</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="21"/>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="19"/>
                 <c:pt idx="0">
-                  <c:v>146</c:v>
+                  <c:v>5.9999999999999609E-2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>150</c:v>
+                  <c:v>4.0000000000000036E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>164</c:v>
+                  <c:v>2.9999999999999805E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>177</c:v>
+                  <c:v>4.0000000000000036E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>192</c:v>
+                  <c:v>4.0000000000000036E-2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>206</c:v>
+                  <c:v>4.9999999999999822E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>219</c:v>
+                  <c:v>6.0000000000000053E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>232</c:v>
+                  <c:v>3.9999999999999591E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>247</c:v>
+                  <c:v>4.0000000000000036E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>258</c:v>
+                  <c:v>4.9999999999999822E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>271</c:v>
+                  <c:v>6.0000000000000497E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>287</c:v>
+                  <c:v>6.0000000000000497E-2</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>305</c:v>
+                  <c:v>4.0000000000000036E-2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>316</c:v>
+                  <c:v>4.0000000000000036E-2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>329</c:v>
+                  <c:v>4.9999999999999822E-2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>343</c:v>
+                  <c:v>4.0000000000000036E-2</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>358</c:v>
+                  <c:v>4.9999999999999822E-2</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>375</c:v>
+                  <c:v>6.0000000000000497E-2</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>376</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>395</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>416</c:v>
+                  <c:v>4.9999999999999822E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2739,7 +2649,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -4609,16 +4519,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>29307</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>590551</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>172182</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>381958</xdr:colOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>343858</xdr:colOff>
       <xdr:row>68</xdr:row>
-      <xdr:rowOff>161542</xdr:rowOff>
+      <xdr:rowOff>123442</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4911,7 +4821,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:S55"/>
+  <dimension ref="B2:T55"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -4929,13 +4839,15 @@
     <col min="13" max="13" width="28.7109375" style="1" customWidth="1"/>
     <col min="14" max="14" width="6.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="8.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.140625" style="1"/>
+    <col min="19" max="19" width="15.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="21.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:18" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:19" s="3" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="9" t="s">
         <v>1</v>
       </c>
@@ -4944,68 +4856,72 @@
       <c r="E2" s="9"/>
       <c r="F2" s="9"/>
       <c r="H2" s="9" t="s">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="I2" s="9"/>
       <c r="J2" s="9"/>
       <c r="K2" s="9"/>
       <c r="L2" s="9"/>
       <c r="N2" s="9" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="O2" s="9"/>
       <c r="P2" s="9"/>
       <c r="Q2" s="9"/>
       <c r="R2" s="9"/>
+      <c r="S2" s="9"/>
     </row>
-    <row r="3" spans="2:18" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
       <c r="B3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>5</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>6</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>0</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="I3" s="4" t="s">
         <v>5</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>6</v>
       </c>
       <c r="J3" s="4" t="s">
         <v>0</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="N3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="O3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="O3" s="4" t="s">
+      <c r="P3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="R3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="P3" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="R3" s="5" t="s">
-        <v>8</v>
+      <c r="S3" s="5" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="4" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B4" s="2">
         <v>2</v>
       </c>
@@ -5040,9 +4956,7 @@
         <f>IF(J4="","",J4/I4)</f>
         <v>66.666666666666671</v>
       </c>
-      <c r="N4" s="2">
-        <v>2</v>
-      </c>
+      <c r="N4" s="2"/>
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
       <c r="Q4" s="2" t="str">
@@ -5050,11 +4964,12 @@
         <v/>
       </c>
       <c r="R4" s="6" t="str">
-        <f>IF(P4="","",P4/O4)</f>
+        <f t="shared" ref="R4:R5" si="0">IF(P4="","",P4/O4/15*1023)</f>
         <v/>
       </c>
+      <c r="S4" s="6"/>
     </row>
-    <row r="5" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B5" s="2">
         <v>2.2000000000000002</v>
       </c>
@@ -5065,11 +4980,11 @@
         <v>190</v>
       </c>
       <c r="E5" s="2">
-        <f t="shared" ref="E5:E24" si="0">IF(C5="","",B5-C5)</f>
+        <f t="shared" ref="E5:E24" si="1">IF(C5="","",B5-C5)</f>
         <v>-0.62999999999999989</v>
       </c>
       <c r="F5" s="6">
-        <f t="shared" ref="F5:F24" si="1">IF(D5="","",D5/C5)</f>
+        <f t="shared" ref="F5:F24" si="2">IF(D5="","",D5/C5)</f>
         <v>67.137809187279146</v>
       </c>
       <c r="H5" s="2">
@@ -5082,28 +4997,27 @@
         <v>150</v>
       </c>
       <c r="K5" s="2">
-        <f t="shared" ref="K5:K24" si="2">H5-I5</f>
+        <f t="shared" ref="K5:K24" si="3">H5-I5</f>
         <v>-5.9999999999999609E-2</v>
       </c>
       <c r="L5" s="6">
-        <f t="shared" ref="L5:L24" si="3">IF(J5="","",J5/I5)</f>
+        <f t="shared" ref="L5:L24" si="4">IF(J5="","",J5/I5)</f>
         <v>66.371681415929203</v>
       </c>
-      <c r="N5" s="2">
-        <v>2.2000000000000002</v>
-      </c>
+      <c r="N5" s="2"/>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
       <c r="Q5" s="2" t="str">
-        <f t="shared" ref="Q5:Q24" si="4">IF(O5="","",N5-O5)</f>
+        <f t="shared" ref="Q5:Q24" si="5">IF(O5="","",N5-O5)</f>
         <v/>
       </c>
       <c r="R5" s="6" t="str">
-        <f t="shared" ref="R5:R24" si="5">IF(P5="","",P5/O5)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
+      <c r="S5" s="6"/>
     </row>
-    <row r="6" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B6" s="2">
         <v>2.4</v>
       </c>
@@ -5114,11 +5028,11 @@
         <v>207</v>
       </c>
       <c r="E6" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.69</v>
       </c>
       <c r="F6" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>66.990291262135926</v>
       </c>
       <c r="H6" s="2">
@@ -5131,28 +5045,36 @@
         <v>164</v>
       </c>
       <c r="K6" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-5.0000000000000266E-2</v>
       </c>
       <c r="L6" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>66.938775510204081</v>
       </c>
       <c r="N6" s="2">
         <v>2.4</v>
       </c>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R6" s="6" t="str">
+      <c r="O6" s="2">
+        <v>2.5499999999999998</v>
+      </c>
+      <c r="P6" s="2">
+        <v>2.4900000000000002</v>
+      </c>
+      <c r="Q6" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>-0.14999999999999991</v>
+      </c>
+      <c r="R6" s="6">
+        <f>IF(P6="","",P6/O6/15*1023)</f>
+        <v>66.595294117647072</v>
+      </c>
+      <c r="S6" s="6">
+        <f>O6-P6</f>
+        <v>5.9999999999999609E-2</v>
       </c>
     </row>
-    <row r="7" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B7" s="2">
         <v>2.6</v>
       </c>
@@ -5163,11 +5085,11 @@
         <v>223</v>
       </c>
       <c r="E7" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.73</v>
       </c>
       <c r="F7" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>66.966966966966964</v>
       </c>
       <c r="H7" s="2">
@@ -5180,28 +5102,36 @@
         <v>177</v>
       </c>
       <c r="K7" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-4.0000000000000036E-2</v>
       </c>
       <c r="L7" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.045454545454547</v>
       </c>
       <c r="N7" s="2">
         <v>2.6</v>
       </c>
-      <c r="O7" s="2"/>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R7" s="6" t="str">
+      <c r="O7" s="2">
+        <v>2.5499999999999998</v>
+      </c>
+      <c r="P7" s="2">
+        <v>2.5099999999999998</v>
+      </c>
+      <c r="Q7" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>5.0000000000000266E-2</v>
+      </c>
+      <c r="R7" s="6">
+        <f t="shared" ref="R7:R24" si="6">IF(P7="","",P7/O7/15*1023)</f>
+        <v>67.130196078431368</v>
+      </c>
+      <c r="S7" s="6">
+        <f t="shared" ref="S7:S24" si="7">O7-P7</f>
+        <v>4.0000000000000036E-2</v>
       </c>
     </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B8" s="2">
         <v>2.8</v>
       </c>
@@ -5212,11 +5142,11 @@
         <v>237</v>
       </c>
       <c r="E8" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.7200000000000002</v>
       </c>
       <c r="F8" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.329545454545453</v>
       </c>
       <c r="H8" s="2">
@@ -5229,28 +5159,36 @@
         <v>192</v>
       </c>
       <c r="K8" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-6.0000000000000053E-2</v>
       </c>
       <c r="L8" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.132867132867133</v>
       </c>
       <c r="N8" s="2">
         <v>2.8</v>
       </c>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R8" s="6" t="str">
+      <c r="O8" s="2">
+        <v>2.76</v>
+      </c>
+      <c r="P8" s="2">
+        <v>2.73</v>
+      </c>
+      <c r="Q8" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>4.0000000000000036E-2</v>
+      </c>
+      <c r="R8" s="6">
+        <f t="shared" si="6"/>
+        <v>67.458695652173915</v>
+      </c>
+      <c r="S8" s="6">
+        <f t="shared" si="7"/>
+        <v>2.9999999999999805E-2</v>
       </c>
     </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B9" s="2">
         <v>3</v>
       </c>
@@ -5261,11 +5199,11 @@
         <v>253</v>
       </c>
       <c r="E9" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.75999999999999979</v>
       </c>
       <c r="F9" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.287234042553195</v>
       </c>
       <c r="H9" s="2">
@@ -5278,28 +5216,36 @@
         <v>206</v>
       </c>
       <c r="K9" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-6.999999999999984E-2</v>
       </c>
       <c r="L9" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.100977198697066</v>
       </c>
       <c r="N9" s="2">
         <v>3</v>
       </c>
-      <c r="O9" s="2"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R9" s="6" t="str">
+      <c r="O9" s="2">
+        <v>2.94</v>
+      </c>
+      <c r="P9" s="2">
+        <v>2.9</v>
+      </c>
+      <c r="Q9" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>6.0000000000000053E-2</v>
+      </c>
+      <c r="R9" s="6">
+        <f t="shared" si="6"/>
+        <v>67.27210884353741</v>
+      </c>
+      <c r="S9" s="6">
+        <f t="shared" si="7"/>
+        <v>4.0000000000000036E-2</v>
       </c>
     </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B10" s="2">
         <v>3.2</v>
       </c>
@@ -5310,11 +5256,11 @@
         <v>265</v>
       </c>
       <c r="E10" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.73999999999999977</v>
       </c>
       <c r="F10" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.258883248730967</v>
       </c>
       <c r="H10" s="2">
@@ -5327,28 +5273,36 @@
         <v>219</v>
       </c>
       <c r="K10" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-6.999999999999984E-2</v>
       </c>
       <c r="L10" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>66.972477064220186</v>
       </c>
       <c r="N10" s="2">
         <v>3.2</v>
       </c>
-      <c r="O10" s="2"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R10" s="6" t="str">
+      <c r="O10" s="2">
+        <v>3.16</v>
+      </c>
+      <c r="P10" s="2">
+        <v>3.12</v>
+      </c>
+      <c r="Q10" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>4.0000000000000036E-2</v>
+      </c>
+      <c r="R10" s="6">
+        <f t="shared" si="6"/>
+        <v>67.336708860759501</v>
+      </c>
+      <c r="S10" s="6">
+        <f t="shared" si="7"/>
+        <v>4.0000000000000036E-2</v>
       </c>
     </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B11" s="2">
         <v>3.4</v>
       </c>
@@ -5359,11 +5313,11 @@
         <v>276</v>
       </c>
       <c r="E11" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.69999999999999973</v>
       </c>
       <c r="F11" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.317073170731717</v>
       </c>
       <c r="H11" s="2">
@@ -5376,28 +5330,36 @@
         <v>232</v>
       </c>
       <c r="K11" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-5.0000000000000266E-2</v>
       </c>
       <c r="L11" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.246376811594203</v>
       </c>
       <c r="N11" s="2">
         <v>3.4</v>
       </c>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R11" s="6" t="str">
+      <c r="O11" s="2">
+        <v>3.36</v>
+      </c>
+      <c r="P11" s="2">
+        <v>3.31</v>
+      </c>
+      <c r="Q11" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>4.0000000000000036E-2</v>
+      </c>
+      <c r="R11" s="6">
+        <f t="shared" si="6"/>
+        <v>67.185119047619054</v>
+      </c>
+      <c r="S11" s="6">
+        <f t="shared" si="7"/>
+        <v>4.9999999999999822E-2</v>
       </c>
     </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B12" s="2">
         <v>3.6</v>
       </c>
@@ -5408,11 +5370,11 @@
         <v>288</v>
       </c>
       <c r="E12" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.66999999999999948</v>
       </c>
       <c r="F12" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.44730679156909</v>
       </c>
       <c r="H12" s="2">
@@ -5425,28 +5387,36 @@
         <v>247</v>
       </c>
       <c r="K12" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-8.0000000000000071E-2</v>
       </c>
       <c r="L12" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.119565217391298</v>
       </c>
       <c r="N12" s="2">
         <v>3.6</v>
       </c>
-      <c r="O12" s="2"/>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R12" s="6" t="str">
+      <c r="O12" s="2">
+        <v>3.56</v>
+      </c>
+      <c r="P12" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="Q12" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>4.0000000000000036E-2</v>
+      </c>
+      <c r="R12" s="6">
+        <f t="shared" si="6"/>
+        <v>67.050561797752806</v>
+      </c>
+      <c r="S12" s="6">
+        <f t="shared" si="7"/>
+        <v>6.0000000000000053E-2</v>
       </c>
     </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B13" s="2">
         <v>3.8</v>
       </c>
@@ -5457,11 +5427,11 @@
         <v>297</v>
       </c>
       <c r="E13" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.60000000000000053</v>
       </c>
       <c r="F13" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.5</v>
       </c>
       <c r="H13" s="2">
@@ -5474,28 +5444,36 @@
         <v>258</v>
       </c>
       <c r="K13" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-4.0000000000000036E-2</v>
       </c>
       <c r="L13" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.1875</v>
       </c>
       <c r="N13" s="2">
         <v>3.8</v>
       </c>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R13" s="6" t="str">
+      <c r="O13" s="2">
+        <v>3.76</v>
+      </c>
+      <c r="P13" s="2">
+        <v>3.72</v>
+      </c>
+      <c r="Q13" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>4.0000000000000036E-2</v>
+      </c>
+      <c r="R13" s="6">
+        <f t="shared" si="6"/>
+        <v>67.474468085106395</v>
+      </c>
+      <c r="S13" s="6">
+        <f t="shared" si="7"/>
+        <v>3.9999999999999591E-2</v>
       </c>
     </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B14" s="2">
         <v>4</v>
       </c>
@@ -5506,11 +5484,11 @@
         <v>307</v>
       </c>
       <c r="E14" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.54</v>
       </c>
       <c r="F14" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.621145374449341</v>
       </c>
       <c r="H14" s="2">
@@ -5523,28 +5501,36 @@
         <v>271</v>
       </c>
       <c r="K14" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-4.0000000000000036E-2</v>
       </c>
       <c r="L14" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.079207920792072</v>
       </c>
       <c r="N14" s="2">
         <v>4</v>
       </c>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R14" s="6" t="str">
+      <c r="O14" s="2">
+        <v>3.94</v>
+      </c>
+      <c r="P14" s="2">
+        <v>3.9</v>
+      </c>
+      <c r="Q14" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>6.0000000000000053E-2</v>
+      </c>
+      <c r="R14" s="6">
+        <f t="shared" si="6"/>
+        <v>67.507614213197968</v>
+      </c>
+      <c r="S14" s="6">
+        <f t="shared" si="7"/>
+        <v>4.0000000000000036E-2</v>
       </c>
     </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B15" s="2">
         <v>4.2</v>
       </c>
@@ -5555,11 +5541,11 @@
         <v>317</v>
       </c>
       <c r="E15" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.5</v>
       </c>
       <c r="F15" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.446808510638292</v>
       </c>
       <c r="H15" s="2">
@@ -5572,28 +5558,36 @@
         <v>287</v>
       </c>
       <c r="K15" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-6.9999999999999396E-2</v>
       </c>
       <c r="L15" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.21311475409837</v>
       </c>
       <c r="N15" s="2">
         <v>4.2</v>
       </c>
-      <c r="O15" s="2"/>
-      <c r="P15" s="2"/>
-      <c r="Q15" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R15" s="6" t="str">
+      <c r="O15" s="2">
+        <v>4.21</v>
+      </c>
+      <c r="P15" s="2">
+        <v>4.16</v>
+      </c>
+      <c r="Q15" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>-9.9999999999997868E-3</v>
+      </c>
+      <c r="R15" s="6">
+        <f t="shared" si="6"/>
+        <v>67.390023752969128</v>
+      </c>
+      <c r="S15" s="6">
+        <f t="shared" si="7"/>
+        <v>4.9999999999999822E-2</v>
       </c>
     </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:19" x14ac:dyDescent="0.2">
       <c r="B16" s="2">
         <v>4.4000000000000004</v>
       </c>
@@ -5604,11 +5598,11 @@
         <v>323</v>
       </c>
       <c r="E16" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.38999999999999968</v>
       </c>
       <c r="F16" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.432150313152405</v>
       </c>
       <c r="H16" s="2">
@@ -5621,28 +5615,36 @@
         <v>305</v>
       </c>
       <c r="K16" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-0.13999999999999968</v>
       </c>
       <c r="L16" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.180616740088112</v>
       </c>
       <c r="N16" s="2">
         <v>4.4000000000000004</v>
       </c>
-      <c r="O16" s="2"/>
-      <c r="P16" s="2"/>
-      <c r="Q16" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R16" s="6" t="str">
+      <c r="O16" s="2">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="P16" s="2">
+        <v>4.34</v>
+      </c>
+      <c r="Q16" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="R16" s="6">
+        <f t="shared" si="6"/>
+        <v>67.27</v>
+      </c>
+      <c r="S16" s="6">
+        <f t="shared" si="7"/>
+        <v>6.0000000000000497E-2</v>
       </c>
     </row>
-    <row r="17" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B17" s="2">
         <v>4.5999999999999996</v>
       </c>
@@ -5653,11 +5655,11 @@
         <v>336</v>
       </c>
       <c r="E17" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.38000000000000078</v>
       </c>
       <c r="F17" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.46987951807229</v>
       </c>
       <c r="H17" s="2">
@@ -5670,28 +5672,36 @@
         <v>316</v>
       </c>
       <c r="K17" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-0.10000000000000053</v>
       </c>
       <c r="L17" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.234042553191486</v>
       </c>
       <c r="N17" s="2">
         <v>4.5999999999999996</v>
       </c>
-      <c r="O17" s="2"/>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R17" s="6" t="str">
+      <c r="O17" s="2">
+        <v>4.62</v>
+      </c>
+      <c r="P17" s="2">
+        <v>4.5599999999999996</v>
+      </c>
+      <c r="Q17" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>-2.0000000000000462E-2</v>
+      </c>
+      <c r="R17" s="6">
+        <f t="shared" si="6"/>
+        <v>67.314285714285703</v>
+      </c>
+      <c r="S17" s="6">
+        <f t="shared" si="7"/>
+        <v>6.0000000000000497E-2</v>
       </c>
     </row>
-    <row r="18" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B18" s="2">
         <v>4.8</v>
       </c>
@@ -5702,11 +5712,11 @@
         <v>343</v>
       </c>
       <c r="E18" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.28000000000000025</v>
       </c>
       <c r="F18" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.519685039370074</v>
       </c>
       <c r="H18" s="2">
@@ -5719,28 +5729,36 @@
         <v>329</v>
       </c>
       <c r="K18" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-8.0000000000000071E-2</v>
       </c>
       <c r="L18" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.418032786885249</v>
       </c>
       <c r="N18" s="2">
         <v>4.8</v>
       </c>
-      <c r="O18" s="2"/>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R18" s="6" t="str">
+      <c r="O18" s="2">
+        <v>4.79</v>
+      </c>
+      <c r="P18" s="2">
+        <v>4.75</v>
+      </c>
+      <c r="Q18" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>9.9999999999997868E-3</v>
+      </c>
+      <c r="R18" s="6">
+        <f t="shared" si="6"/>
+        <v>67.630480167014611</v>
+      </c>
+      <c r="S18" s="6">
+        <f t="shared" si="7"/>
+        <v>4.0000000000000036E-2</v>
       </c>
     </row>
-    <row r="19" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B19" s="2">
         <v>5</v>
       </c>
@@ -5751,11 +5769,11 @@
         <v>351</v>
       </c>
       <c r="E19" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.20000000000000018</v>
       </c>
       <c r="F19" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.5</v>
       </c>
       <c r="H19" s="2">
@@ -5768,28 +5786,36 @@
         <v>343</v>
       </c>
       <c r="K19" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-8.0000000000000071E-2</v>
       </c>
       <c r="L19" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.519685039370074</v>
       </c>
       <c r="N19" s="2">
         <v>5</v>
       </c>
-      <c r="O19" s="2"/>
-      <c r="P19" s="2"/>
-      <c r="Q19" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R19" s="6" t="str">
+      <c r="O19" s="2">
+        <v>4.9800000000000004</v>
+      </c>
+      <c r="P19" s="2">
+        <v>4.9400000000000004</v>
+      </c>
+      <c r="Q19" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>1.9999999999999574E-2</v>
+      </c>
+      <c r="R19" s="6">
+        <f t="shared" si="6"/>
+        <v>67.652208835341369</v>
+      </c>
+      <c r="S19" s="6">
+        <f t="shared" si="7"/>
+        <v>4.0000000000000036E-2</v>
       </c>
     </row>
-    <row r="20" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B20" s="2">
         <v>5.2</v>
       </c>
@@ -5800,11 +5826,11 @@
         <v>359</v>
       </c>
       <c r="E20" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.12000000000000011</v>
       </c>
       <c r="F20" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.481203007518786</v>
       </c>
       <c r="H20" s="2">
@@ -5817,28 +5843,36 @@
         <v>358</v>
       </c>
       <c r="K20" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-0.12000000000000011</v>
       </c>
       <c r="L20" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.293233082706763</v>
       </c>
       <c r="N20" s="2">
         <v>5.2</v>
       </c>
-      <c r="O20" s="2"/>
-      <c r="P20" s="2"/>
-      <c r="Q20" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R20" s="6" t="str">
+      <c r="O20" s="2">
+        <v>5.21</v>
+      </c>
+      <c r="P20" s="2">
+        <v>5.16</v>
+      </c>
+      <c r="Q20" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>-9.9999999999997868E-3</v>
+      </c>
+      <c r="R20" s="6">
+        <f t="shared" si="6"/>
+        <v>67.545489443378131</v>
+      </c>
+      <c r="S20" s="6">
+        <f t="shared" si="7"/>
+        <v>4.9999999999999822E-2</v>
       </c>
     </row>
-    <row r="21" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B21" s="2">
         <v>5.4</v>
       </c>
@@ -5849,11 +5883,11 @@
         <v>368</v>
       </c>
       <c r="E21" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-4.0000000000000036E-2</v>
       </c>
       <c r="F21" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.647058823529406</v>
       </c>
       <c r="H21" s="2">
@@ -5866,28 +5900,36 @@
         <v>375</v>
       </c>
       <c r="K21" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-0.16999999999999993</v>
       </c>
       <c r="L21" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.324955116696586</v>
       </c>
       <c r="N21" s="2">
         <v>5.4</v>
       </c>
-      <c r="O21" s="2"/>
-      <c r="P21" s="2"/>
-      <c r="Q21" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R21" s="6" t="str">
+      <c r="O21" s="2">
+        <v>5.45</v>
+      </c>
+      <c r="P21" s="2">
+        <v>5.41</v>
+      </c>
+      <c r="Q21" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>-4.9999999999999822E-2</v>
+      </c>
+      <c r="R21" s="6">
+        <f t="shared" si="6"/>
+        <v>67.699449541284395</v>
+      </c>
+      <c r="S21" s="6">
+        <f t="shared" si="7"/>
+        <v>4.0000000000000036E-2</v>
       </c>
     </row>
-    <row r="22" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B22" s="2">
         <v>5.6</v>
       </c>
@@ -5898,11 +5940,11 @@
         <v>377</v>
       </c>
       <c r="E22" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.9999999999999361E-2</v>
       </c>
       <c r="F22" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.684021543985637</v>
       </c>
       <c r="H22" s="2">
@@ -5915,28 +5957,36 @@
         <v>376</v>
       </c>
       <c r="K22" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2.9999999999999361E-2</v>
       </c>
       <c r="L22" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.504488330341104</v>
       </c>
       <c r="N22" s="2">
         <v>5.6</v>
       </c>
-      <c r="O22" s="2"/>
-      <c r="P22" s="2"/>
-      <c r="Q22" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R22" s="6" t="str">
+      <c r="O22" s="2">
+        <v>5.58</v>
+      </c>
+      <c r="P22" s="2">
+        <v>5.53</v>
+      </c>
+      <c r="Q22" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>1.9999999999999574E-2</v>
+      </c>
+      <c r="R22" s="6">
+        <f t="shared" si="6"/>
+        <v>67.588888888888889</v>
+      </c>
+      <c r="S22" s="6">
+        <f t="shared" si="7"/>
+        <v>4.9999999999999822E-2</v>
       </c>
     </row>
-    <row r="23" spans="2:19" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:20" ht="15.75" x14ac:dyDescent="0.2">
       <c r="B23" s="2">
         <v>5.8</v>
       </c>
@@ -5947,15 +5997,15 @@
         <v>377</v>
       </c>
       <c r="E23" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.22999999999999954</v>
       </c>
       <c r="F23" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.684021543985637</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H23" s="2">
         <v>5.8</v>
@@ -5967,31 +6017,42 @@
         <v>395</v>
       </c>
       <c r="K23" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-6.0000000000000497E-2</v>
       </c>
       <c r="L23" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.406143344709889</v>
       </c>
       <c r="M23" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="N23" s="2">
         <v>5.8</v>
       </c>
-      <c r="O23" s="2"/>
-      <c r="P23" s="2"/>
-      <c r="Q23" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R23" s="6" t="str">
+      <c r="O23" s="2">
+        <v>5.87</v>
+      </c>
+      <c r="P23" s="2">
+        <v>5.81</v>
+      </c>
+      <c r="Q23" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>-7.0000000000000284E-2</v>
+      </c>
+      <c r="R23" s="6">
+        <f t="shared" si="6"/>
+        <v>67.502896081771709</v>
+      </c>
+      <c r="S23" s="6">
+        <f t="shared" si="7"/>
+        <v>6.0000000000000497E-2</v>
+      </c>
+      <c r="T23" s="4" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="24" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B24" s="2">
         <v>6</v>
       </c>
@@ -6002,11 +6063,11 @@
         <v>418</v>
       </c>
       <c r="E24" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-0.17999999999999972</v>
       </c>
       <c r="F24" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>67.637540453074436</v>
       </c>
       <c r="G24" s="2">
@@ -6023,11 +6084,11 @@
         <v>416</v>
       </c>
       <c r="K24" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-0.17999999999999972</v>
       </c>
       <c r="L24" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>67.313915857605181</v>
       </c>
       <c r="M24" s="2">
@@ -6037,28 +6098,40 @@
       <c r="N24" s="2">
         <v>6</v>
       </c>
-      <c r="O24" s="2"/>
-      <c r="P24" s="2"/>
-      <c r="Q24" s="2" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="R24" s="6" t="str">
+      <c r="O24" s="2">
+        <v>6.02</v>
+      </c>
+      <c r="P24" s="2">
+        <v>5.97</v>
+      </c>
+      <c r="Q24" s="2">
         <f t="shared" si="5"/>
-        <v/>
+        <v>-1.9999999999999574E-2</v>
+      </c>
+      <c r="R24" s="6">
+        <f t="shared" si="6"/>
+        <v>67.633554817275751</v>
+      </c>
+      <c r="S24" s="6">
+        <f t="shared" si="7"/>
+        <v>4.9999999999999822E-2</v>
+      </c>
+      <c r="T24" s="6">
+        <f>AVERAGE(S4:S24)</f>
+        <v>4.7368421052631574E-2</v>
       </c>
     </row>
-    <row r="31" spans="2:19" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:20" x14ac:dyDescent="0.2">
       <c r="S31" s="8" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="49" spans="8:9" ht="15" x14ac:dyDescent="0.2">
       <c r="H49" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="I49" s="7" t="s">
         <v>3</v>
-      </c>
-      <c r="I49" s="7" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="50" spans="8:9" x14ac:dyDescent="0.2">
@@ -6081,10 +6154,10 @@
     </row>
     <row r="53" spans="8:9" ht="15" x14ac:dyDescent="0.2">
       <c r="H53" s="7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I53" s="7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="54" spans="8:9" x14ac:dyDescent="0.2">
@@ -6097,7 +6170,7 @@
     </row>
     <row r="55" spans="8:9" ht="15" x14ac:dyDescent="0.2">
       <c r="H55" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I55" s="2">
         <f>I54/H54</f>
@@ -6108,156 +6181,10 @@
   <mergeCells count="3">
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="H2:L2"/>
-    <mergeCell ref="N2:R2"/>
+    <mergeCell ref="N2:S2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C187DCCE-8E32-44A3-9556-14C14F1C388A}">
-  <dimension ref="B3:C24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="3" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="2">
-        <v>0.72499999999999998</v>
-      </c>
-      <c r="C4" s="2">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="2"/>
-      <c r="C5" s="2">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="2"/>
-      <c r="C6" s="2">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="2"/>
-      <c r="C7" s="2">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="2"/>
-      <c r="C8" s="2">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="2"/>
-      <c r="C9" s="2">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="2"/>
-      <c r="C10" s="2">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="2"/>
-      <c r="C11" s="2">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B12" s="2"/>
-      <c r="C12" s="2">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B13" s="2"/>
-      <c r="C13" s="2">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B14" s="2"/>
-      <c r="C14" s="2">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B15" s="2"/>
-      <c r="C15" s="2">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B16" s="2"/>
-      <c r="C16" s="2">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B17" s="2"/>
-      <c r="C17" s="2">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B18" s="2"/>
-      <c r="C18" s="2">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B19" s="2"/>
-      <c r="C19" s="2">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B20" s="2"/>
-      <c r="C20" s="2">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B21" s="2"/>
-      <c r="C21" s="2">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B22" s="2"/>
-      <c r="C22" s="2">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B23" s="2"/>
-      <c r="C23" s="2">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B24" s="2"/>
-      <c r="C24" s="2">
-        <v>416</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Finished README, updated Data.xlsx with updated feedback loop data. Added images. Added Altium project file.
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a4fd901eb976e385/Desktop/Power Supply/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="406" documentId="11_F25DC773A252ABDACC10487EC95C72D65BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D58204A0-B3F4-4E5E-ADDA-C6F9C32CB9FD}"/>
+  <xr:revisionPtr revIDLastSave="470" documentId="11_F25DC773A252ABDACC10487EC95C72D65BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C915E04-ED5E-4376-BD58-0B1754BAD2E1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,8 +35,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="18">
   <si>
     <t>Vsense</t>
   </si>
@@ -60,9 +82,6 @@
   </si>
   <si>
     <t>Error</t>
-  </si>
-  <si>
-    <t>Go into graph filters to bring back 256 tap</t>
   </si>
   <si>
     <t>Avg. Error</t>
@@ -654,6 +673,9 @@
         <c:ser>
           <c:idx val="2"/>
           <c:order val="2"/>
+          <c:tx>
+            <c:v>Feedback (256 Tap)</c:v>
+          </c:tx>
           <c:spPr>
             <a:ln w="25400" cap="rnd">
               <a:noFill/>
@@ -749,61 +771,61 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
                 <c:pt idx="0">
-                  <c:v>-0.14999999999999991</c:v>
+                  <c:v>-4.9999999999998934E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.0000000000000266E-2</c:v>
+                  <c:v>-4.0000000000000036E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.0000000000000036E-2</c:v>
+                  <c:v>-3.0000000000000249E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>6.0000000000000053E-2</c:v>
+                  <c:v>-2.0000000000000018E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.0000000000000036E-2</c:v>
+                  <c:v>-1.7999999999999794E-2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4.0000000000000036E-2</c:v>
+                  <c:v>7.0000000000001172E-3</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>4.0000000000000036E-2</c:v>
+                  <c:v>9.9999999999988987E-4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.0000000000000036E-2</c:v>
+                  <c:v>-6.0000000000002274E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>6.0000000000000053E-2</c:v>
+                  <c:v>1.9999999999997797E-3</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-9.9999999999997868E-3</c:v>
+                  <c:v>-1.4000000000000234E-2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>-3.9999999999995595E-3</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-2.0000000000000462E-2</c:v>
+                  <c:v>-2.5000000000000355E-2</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>9.9999999999997868E-3</c:v>
+                  <c:v>3.9999999999995595E-3</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1.9999999999999574E-2</c:v>
+                  <c:v>1.1000000000000121E-2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-9.9999999999997868E-3</c:v>
+                  <c:v>-1.499999999999968E-2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-4.9999999999999822E-2</c:v>
+                  <c:v>-5.6999999999999496E-2</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1.9999999999999574E-2</c:v>
+                  <c:v>1.1999999999999567E-2</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-7.0000000000000284E-2</c:v>
+                  <c:v>-7.5000000000000178E-2</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-1.9999999999999574E-2</c:v>
+                  <c:v>-3.2000000000000028E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -976,7 +998,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-AU"/>
-                  <a:t>Target</a:t>
+                  <a:t>Tracking</a:t>
                 </a:r>
                 <a:r>
                   <a:rPr lang="en-AU" baseline="0"/>
@@ -1706,61 +1728,61 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="19"/>
                 <c:pt idx="0">
-                  <c:v>66.595294117647072</c:v>
+                  <c:v>68.341787941787956</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>67.130196078431368</c:v>
+                  <c:v>68.095238095238102</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>67.458695652173915</c:v>
+                  <c:v>67.718021201413421</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>67.27210884353741</c:v>
+                  <c:v>67.974172185430461</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>67.336708860759501</c:v>
+                  <c:v>68.242386575512739</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>67.185119047619054</c:v>
+                  <c:v>68.54170350722076</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>67.050561797752806</c:v>
+                  <c:v>68.408446790775216</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>67.474468085106395</c:v>
+                  <c:v>68.092485549132945</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>67.507614213197968</c:v>
+                  <c:v>67.89294647323662</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>67.390023752969128</c:v>
+                  <c:v>68.135263407688655</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>67.27</c:v>
+                  <c:v>67.983197093551311</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>67.314285714285703</c:v>
+                  <c:v>68.126270270270268</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>67.630480167014611</c:v>
+                  <c:v>68.541284403669721</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>67.652208835341369</c:v>
+                  <c:v>68.076969332531576</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>67.545489443378131</c:v>
+                  <c:v>66.957622243528292</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>67.699449541284395</c:v>
+                  <c:v>68.112516034451176</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>67.588888888888889</c:v>
+                  <c:v>68.1023622047244</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>67.502896081771709</c:v>
+                  <c:v>68.374127659574469</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>67.633554817275751</c:v>
+                  <c:v>68.064323607427056</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2320,61 +2342,61 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
                 <c:pt idx="0">
-                  <c:v>2.5499999999999998</c:v>
+                  <c:v>2.4049999999999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.5499999999999998</c:v>
+                  <c:v>2.6040000000000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.76</c:v>
+                  <c:v>2.83</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2.94</c:v>
+                  <c:v>3.02</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3.16</c:v>
+                  <c:v>3.218</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3.36</c:v>
+                  <c:v>3.3929999999999998</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>3.56</c:v>
+                  <c:v>3.5990000000000002</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>3.76</c:v>
+                  <c:v>3.806</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3.94</c:v>
+                  <c:v>3.9980000000000002</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4.21</c:v>
+                  <c:v>4.2140000000000004</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>4.4000000000000004</c:v>
+                  <c:v>4.4039999999999999</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>4.62</c:v>
+                  <c:v>4.625</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>4.79</c:v>
+                  <c:v>4.7960000000000003</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>4.9800000000000004</c:v>
+                  <c:v>4.9889999999999999</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>5.21</c:v>
+                  <c:v>5.2149999999999999</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>5.45</c:v>
+                  <c:v>5.4569999999999999</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>5.58</c:v>
+                  <c:v>5.5880000000000001</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>5.87</c:v>
+                  <c:v>5.875</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>6.02</c:v>
+                  <c:v>6.032</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2386,61 +2408,61 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="19"/>
                 <c:pt idx="0">
-                  <c:v>5.9999999999999609E-2</c:v>
+                  <c:v>-5.0000000000003375E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.0000000000000036E-2</c:v>
+                  <c:v>4.0000000000000036E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.9999999999999805E-2</c:v>
+                  <c:v>2.0000000000000018E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4.0000000000000036E-2</c:v>
+                  <c:v>1.0000000000000231E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.0000000000000036E-2</c:v>
+                  <c:v>-2.0000000000002238E-3</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4.9999999999999822E-2</c:v>
+                  <c:v>-1.7000000000000348E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6.0000000000000053E-2</c:v>
+                  <c:v>-1.0999999999999677E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>3.9999999999999591E-2</c:v>
+                  <c:v>6.0000000000002274E-3</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4.0000000000000036E-2</c:v>
+                  <c:v>1.8000000000000238E-2</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4.9999999999999822E-2</c:v>
+                  <c:v>4.0000000000004476E-3</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>6.0000000000000497E-2</c:v>
+                  <c:v>1.4000000000000234E-2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>6.0000000000000497E-2</c:v>
+                  <c:v>4.9999999999998934E-3</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>4.0000000000000036E-2</c:v>
+                  <c:v>-2.4000000000000021E-2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>4.0000000000000036E-2</c:v>
+                  <c:v>8.9999999999994529E-3</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>4.9999999999999822E-2</c:v>
+                  <c:v>9.4999999999999751E-2</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>4.0000000000000036E-2</c:v>
+                  <c:v>6.9999999999996732E-3</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>4.9999999999999822E-2</c:v>
+                  <c:v>8.0000000000000071E-3</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>6.0000000000000497E-2</c:v>
+                  <c:v>-1.499999999999968E-2</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>4.9999999999999822E-2</c:v>
+                  <c:v>1.2000000000000455E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4451,8 +4473,8 @@
       <xdr:rowOff>13898</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>1615109</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>46</xdr:row>
       <xdr:rowOff>157370</xdr:rowOff>
     </xdr:to>
@@ -4481,16 +4503,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>1697933</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>1242</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>393008</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>67917</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>372717</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>1382367</xdr:colOff>
       <xdr:row>46</xdr:row>
-      <xdr:rowOff>140804</xdr:rowOff>
+      <xdr:rowOff>26504</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -4856,14 +4878,14 @@
       <c r="E2" s="9"/>
       <c r="F2" s="9"/>
       <c r="H2" s="9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I2" s="9"/>
       <c r="J2" s="9"/>
       <c r="K2" s="9"/>
       <c r="L2" s="9"/>
       <c r="N2" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="O2" s="9"/>
       <c r="P2" s="9"/>
@@ -4909,16 +4931,16 @@
         <v>5</v>
       </c>
       <c r="P3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q3" s="5" t="s">
         <v>14</v>
-      </c>
-      <c r="Q3" s="5" t="s">
-        <v>15</v>
       </c>
       <c r="R3" s="5" t="s">
         <v>6</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="2:19" x14ac:dyDescent="0.2">
@@ -5056,22 +5078,22 @@
         <v>2.4</v>
       </c>
       <c r="O6" s="2">
-        <v>2.5499999999999998</v>
+        <v>2.4049999999999998</v>
       </c>
       <c r="P6" s="2">
-        <v>2.4900000000000002</v>
+        <v>2.41</v>
       </c>
       <c r="Q6" s="2">
         <f t="shared" si="5"/>
-        <v>-0.14999999999999991</v>
+        <v>-4.9999999999998934E-3</v>
       </c>
       <c r="R6" s="6">
         <f>IF(P6="","",P6/O6/15*1023)</f>
-        <v>66.595294117647072</v>
+        <v>68.341787941787956</v>
       </c>
       <c r="S6" s="6">
         <f>O6-P6</f>
-        <v>5.9999999999999609E-2</v>
+        <v>-5.0000000000003375E-3</v>
       </c>
     </row>
     <row r="7" spans="2:19" x14ac:dyDescent="0.2">
@@ -5113,22 +5135,22 @@
         <v>2.6</v>
       </c>
       <c r="O7" s="2">
-        <v>2.5499999999999998</v>
+        <v>2.6040000000000001</v>
       </c>
       <c r="P7" s="2">
-        <v>2.5099999999999998</v>
+        <v>2.6</v>
       </c>
       <c r="Q7" s="2">
         <f t="shared" si="5"/>
-        <v>5.0000000000000266E-2</v>
+        <v>-4.0000000000000036E-3</v>
       </c>
       <c r="R7" s="6">
         <f t="shared" ref="R7:R24" si="6">IF(P7="","",P7/O7/15*1023)</f>
-        <v>67.130196078431368</v>
+        <v>68.095238095238102</v>
       </c>
       <c r="S7" s="6">
         <f t="shared" ref="S7:S24" si="7">O7-P7</f>
-        <v>4.0000000000000036E-2</v>
+        <v>4.0000000000000036E-3</v>
       </c>
     </row>
     <row r="8" spans="2:19" x14ac:dyDescent="0.2">
@@ -5170,22 +5192,22 @@
         <v>2.8</v>
       </c>
       <c r="O8" s="2">
-        <v>2.76</v>
+        <v>2.83</v>
       </c>
       <c r="P8" s="2">
-        <v>2.73</v>
+        <v>2.81</v>
       </c>
       <c r="Q8" s="2">
         <f t="shared" si="5"/>
-        <v>4.0000000000000036E-2</v>
+        <v>-3.0000000000000249E-2</v>
       </c>
       <c r="R8" s="6">
         <f t="shared" si="6"/>
-        <v>67.458695652173915</v>
+        <v>67.718021201413421</v>
       </c>
       <c r="S8" s="6">
         <f t="shared" si="7"/>
-        <v>2.9999999999999805E-2</v>
+        <v>2.0000000000000018E-2</v>
       </c>
     </row>
     <row r="9" spans="2:19" x14ac:dyDescent="0.2">
@@ -5227,22 +5249,22 @@
         <v>3</v>
       </c>
       <c r="O9" s="2">
-        <v>2.94</v>
+        <v>3.02</v>
       </c>
       <c r="P9" s="2">
-        <v>2.9</v>
+        <v>3.01</v>
       </c>
       <c r="Q9" s="2">
         <f t="shared" si="5"/>
-        <v>6.0000000000000053E-2</v>
+        <v>-2.0000000000000018E-2</v>
       </c>
       <c r="R9" s="6">
         <f t="shared" si="6"/>
-        <v>67.27210884353741</v>
+        <v>67.974172185430461</v>
       </c>
       <c r="S9" s="6">
         <f t="shared" si="7"/>
-        <v>4.0000000000000036E-2</v>
+        <v>1.0000000000000231E-2</v>
       </c>
     </row>
     <row r="10" spans="2:19" x14ac:dyDescent="0.2">
@@ -5284,22 +5306,22 @@
         <v>3.2</v>
       </c>
       <c r="O10" s="2">
-        <v>3.16</v>
+        <v>3.218</v>
       </c>
       <c r="P10" s="2">
-        <v>3.12</v>
+        <v>3.22</v>
       </c>
       <c r="Q10" s="2">
         <f t="shared" si="5"/>
-        <v>4.0000000000000036E-2</v>
+        <v>-1.7999999999999794E-2</v>
       </c>
       <c r="R10" s="6">
         <f t="shared" si="6"/>
-        <v>67.336708860759501</v>
+        <v>68.242386575512739</v>
       </c>
       <c r="S10" s="6">
         <f t="shared" si="7"/>
-        <v>4.0000000000000036E-2</v>
+        <v>-2.0000000000002238E-3</v>
       </c>
     </row>
     <row r="11" spans="2:19" x14ac:dyDescent="0.2">
@@ -5341,22 +5363,22 @@
         <v>3.4</v>
       </c>
       <c r="O11" s="2">
-        <v>3.36</v>
+        <v>3.3929999999999998</v>
       </c>
       <c r="P11" s="2">
-        <v>3.31</v>
+        <v>3.41</v>
       </c>
       <c r="Q11" s="2">
         <f t="shared" si="5"/>
-        <v>4.0000000000000036E-2</v>
+        <v>7.0000000000001172E-3</v>
       </c>
       <c r="R11" s="6">
         <f t="shared" si="6"/>
-        <v>67.185119047619054</v>
+        <v>68.54170350722076</v>
       </c>
       <c r="S11" s="6">
         <f t="shared" si="7"/>
-        <v>4.9999999999999822E-2</v>
+        <v>-1.7000000000000348E-2</v>
       </c>
     </row>
     <row r="12" spans="2:19" x14ac:dyDescent="0.2">
@@ -5398,22 +5420,22 @@
         <v>3.6</v>
       </c>
       <c r="O12" s="2">
-        <v>3.56</v>
+        <v>3.5990000000000002</v>
       </c>
       <c r="P12" s="2">
-        <v>3.5</v>
+        <v>3.61</v>
       </c>
       <c r="Q12" s="2">
         <f t="shared" si="5"/>
-        <v>4.0000000000000036E-2</v>
+        <v>9.9999999999988987E-4</v>
       </c>
       <c r="R12" s="6">
         <f t="shared" si="6"/>
-        <v>67.050561797752806</v>
+        <v>68.408446790775216</v>
       </c>
       <c r="S12" s="6">
         <f t="shared" si="7"/>
-        <v>6.0000000000000053E-2</v>
+        <v>-1.0999999999999677E-2</v>
       </c>
     </row>
     <row r="13" spans="2:19" x14ac:dyDescent="0.2">
@@ -5455,22 +5477,22 @@
         <v>3.8</v>
       </c>
       <c r="O13" s="2">
-        <v>3.76</v>
+        <v>3.806</v>
       </c>
       <c r="P13" s="2">
-        <v>3.72</v>
+        <v>3.8</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" si="5"/>
-        <v>4.0000000000000036E-2</v>
+        <v>-6.0000000000002274E-3</v>
       </c>
       <c r="R13" s="6">
         <f t="shared" si="6"/>
-        <v>67.474468085106395</v>
+        <v>68.092485549132945</v>
       </c>
       <c r="S13" s="6">
         <f t="shared" si="7"/>
-        <v>3.9999999999999591E-2</v>
+        <v>6.0000000000002274E-3</v>
       </c>
     </row>
     <row r="14" spans="2:19" x14ac:dyDescent="0.2">
@@ -5512,22 +5534,22 @@
         <v>4</v>
       </c>
       <c r="O14" s="2">
-        <v>3.94</v>
+        <v>3.9980000000000002</v>
       </c>
       <c r="P14" s="2">
-        <v>3.9</v>
+        <v>3.98</v>
       </c>
       <c r="Q14" s="2">
         <f t="shared" si="5"/>
-        <v>6.0000000000000053E-2</v>
+        <v>1.9999999999997797E-3</v>
       </c>
       <c r="R14" s="6">
         <f t="shared" si="6"/>
-        <v>67.507614213197968</v>
+        <v>67.89294647323662</v>
       </c>
       <c r="S14" s="6">
         <f t="shared" si="7"/>
-        <v>4.0000000000000036E-2</v>
+        <v>1.8000000000000238E-2</v>
       </c>
     </row>
     <row r="15" spans="2:19" x14ac:dyDescent="0.2">
@@ -5569,22 +5591,22 @@
         <v>4.2</v>
       </c>
       <c r="O15" s="2">
+        <v>4.2140000000000004</v>
+      </c>
+      <c r="P15" s="2">
         <v>4.21</v>
-      </c>
-      <c r="P15" s="2">
-        <v>4.16</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" si="5"/>
-        <v>-9.9999999999997868E-3</v>
+        <v>-1.4000000000000234E-2</v>
       </c>
       <c r="R15" s="6">
         <f t="shared" si="6"/>
-        <v>67.390023752969128</v>
+        <v>68.135263407688655</v>
       </c>
       <c r="S15" s="6">
         <f t="shared" si="7"/>
-        <v>4.9999999999999822E-2</v>
+        <v>4.0000000000004476E-3</v>
       </c>
     </row>
     <row r="16" spans="2:19" x14ac:dyDescent="0.2">
@@ -5626,22 +5648,22 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="O16" s="2">
-        <v>4.4000000000000004</v>
+        <v>4.4039999999999999</v>
       </c>
       <c r="P16" s="2">
-        <v>4.34</v>
+        <v>4.3899999999999997</v>
       </c>
       <c r="Q16" s="2">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>-3.9999999999995595E-3</v>
       </c>
       <c r="R16" s="6">
         <f t="shared" si="6"/>
-        <v>67.27</v>
+        <v>67.983197093551311</v>
       </c>
       <c r="S16" s="6">
         <f t="shared" si="7"/>
-        <v>6.0000000000000497E-2</v>
+        <v>1.4000000000000234E-2</v>
       </c>
     </row>
     <row r="17" spans="2:20" x14ac:dyDescent="0.2">
@@ -5683,22 +5705,22 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="O17" s="2">
+        <v>4.625</v>
+      </c>
+      <c r="P17" s="2">
         <v>4.62</v>
-      </c>
-      <c r="P17" s="2">
-        <v>4.5599999999999996</v>
       </c>
       <c r="Q17" s="2">
         <f t="shared" si="5"/>
-        <v>-2.0000000000000462E-2</v>
+        <v>-2.5000000000000355E-2</v>
       </c>
       <c r="R17" s="6">
         <f t="shared" si="6"/>
-        <v>67.314285714285703</v>
+        <v>68.126270270270268</v>
       </c>
       <c r="S17" s="6">
         <f t="shared" si="7"/>
-        <v>6.0000000000000497E-2</v>
+        <v>4.9999999999998934E-3</v>
       </c>
     </row>
     <row r="18" spans="2:20" x14ac:dyDescent="0.2">
@@ -5740,22 +5762,22 @@
         <v>4.8</v>
       </c>
       <c r="O18" s="2">
-        <v>4.79</v>
+        <v>4.7960000000000003</v>
       </c>
       <c r="P18" s="2">
-        <v>4.75</v>
+        <v>4.82</v>
       </c>
       <c r="Q18" s="2">
         <f t="shared" si="5"/>
-        <v>9.9999999999997868E-3</v>
+        <v>3.9999999999995595E-3</v>
       </c>
       <c r="R18" s="6">
         <f t="shared" si="6"/>
-        <v>67.630480167014611</v>
+        <v>68.541284403669721</v>
       </c>
       <c r="S18" s="6">
         <f t="shared" si="7"/>
-        <v>4.0000000000000036E-2</v>
+        <v>-2.4000000000000021E-2</v>
       </c>
     </row>
     <row r="19" spans="2:20" x14ac:dyDescent="0.2">
@@ -5797,22 +5819,22 @@
         <v>5</v>
       </c>
       <c r="O19" s="2">
+        <v>4.9889999999999999</v>
+      </c>
+      <c r="P19" s="2">
         <v>4.9800000000000004</v>
-      </c>
-      <c r="P19" s="2">
-        <v>4.9400000000000004</v>
       </c>
       <c r="Q19" s="2">
         <f t="shared" si="5"/>
-        <v>1.9999999999999574E-2</v>
+        <v>1.1000000000000121E-2</v>
       </c>
       <c r="R19" s="6">
         <f t="shared" si="6"/>
-        <v>67.652208835341369</v>
+        <v>68.076969332531576</v>
       </c>
       <c r="S19" s="6">
         <f t="shared" si="7"/>
-        <v>4.0000000000000036E-2</v>
+        <v>8.9999999999994529E-3</v>
       </c>
     </row>
     <row r="20" spans="2:20" x14ac:dyDescent="0.2">
@@ -5854,25 +5876,25 @@
         <v>5.2</v>
       </c>
       <c r="O20" s="2">
-        <v>5.21</v>
+        <v>5.2149999999999999</v>
       </c>
       <c r="P20" s="2">
-        <v>5.16</v>
+        <v>5.12</v>
       </c>
       <c r="Q20" s="2">
         <f t="shared" si="5"/>
-        <v>-9.9999999999997868E-3</v>
+        <v>-1.499999999999968E-2</v>
       </c>
       <c r="R20" s="6">
         <f t="shared" si="6"/>
-        <v>67.545489443378131</v>
+        <v>66.957622243528292</v>
       </c>
       <c r="S20" s="6">
         <f t="shared" si="7"/>
-        <v>4.9999999999999822E-2</v>
+        <v>9.4999999999999751E-2</v>
       </c>
     </row>
-    <row r="21" spans="2:20" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:20" ht="15.75" x14ac:dyDescent="0.2">
       <c r="B21" s="2">
         <v>5.4</v>
       </c>
@@ -5911,22 +5933,25 @@
         <v>5.4</v>
       </c>
       <c r="O21" s="2">
+        <v>5.4569999999999999</v>
+      </c>
+      <c r="P21" s="2">
         <v>5.45</v>
-      </c>
-      <c r="P21" s="2">
-        <v>5.41</v>
       </c>
       <c r="Q21" s="2">
         <f t="shared" si="5"/>
-        <v>-4.9999999999999822E-2</v>
+        <v>-5.6999999999999496E-2</v>
       </c>
       <c r="R21" s="6">
         <f t="shared" si="6"/>
-        <v>67.699449541284395</v>
+        <v>68.112516034451176</v>
       </c>
       <c r="S21" s="6">
         <f t="shared" si="7"/>
-        <v>4.0000000000000036E-2</v>
+        <v>6.9999999999996732E-3</v>
+      </c>
+      <c r="T21" s="4" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="22" spans="2:20" x14ac:dyDescent="0.2">
@@ -5968,22 +5993,26 @@
         <v>5.6</v>
       </c>
       <c r="O22" s="2">
+        <v>5.5880000000000001</v>
+      </c>
+      <c r="P22" s="2">
         <v>5.58</v>
-      </c>
-      <c r="P22" s="2">
-        <v>5.53</v>
       </c>
       <c r="Q22" s="2">
         <f t="shared" si="5"/>
-        <v>1.9999999999999574E-2</v>
+        <v>1.1999999999999567E-2</v>
       </c>
       <c r="R22" s="6">
         <f t="shared" si="6"/>
-        <v>67.588888888888889</v>
+        <v>68.1023622047244</v>
       </c>
       <c r="S22" s="6">
         <f t="shared" si="7"/>
-        <v>4.9999999999999822E-2</v>
+        <v>8.0000000000000071E-3</v>
+      </c>
+      <c r="T22" s="6">
+        <f>AVERAGE(S4:S24)</f>
+        <v>7.2631578947368602E-3</v>
       </c>
     </row>
     <row r="23" spans="2:20" ht="15.75" x14ac:dyDescent="0.2">
@@ -6005,7 +6034,7 @@
         <v>67.684021543985637</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H23" s="2">
         <v>5.8</v>
@@ -6025,31 +6054,31 @@
         <v>67.406143344709889</v>
       </c>
       <c r="M23" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N23" s="2">
         <v>5.8</v>
       </c>
       <c r="O23" s="2">
-        <v>5.87</v>
+        <v>5.875</v>
       </c>
       <c r="P23" s="2">
-        <v>5.81</v>
+        <v>5.89</v>
       </c>
       <c r="Q23" s="2">
         <f t="shared" si="5"/>
-        <v>-7.0000000000000284E-2</v>
+        <v>-7.5000000000000178E-2</v>
       </c>
       <c r="R23" s="6">
         <f t="shared" si="6"/>
-        <v>67.502896081771709</v>
+        <v>68.374127659574469</v>
       </c>
       <c r="S23" s="6">
         <f t="shared" si="7"/>
-        <v>6.0000000000000497E-2</v>
+        <v>-1.499999999999968E-2</v>
       </c>
       <c r="T23" s="4" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="2:20" x14ac:dyDescent="0.2">
@@ -6091,40 +6120,38 @@
         <f t="shared" si="4"/>
         <v>67.313915857605181</v>
       </c>
-      <c r="M24" s="2">
-        <f>AVERAGE(K4:K24)</f>
-        <v>-8.1904761904761939E-2</v>
+      <c r="M24" s="2" cm="1">
+        <f t="array" ref="M24">SUMPRODUCT(ABS(K4:K24))/COUNT(K4:K24)</f>
+        <v>8.4761904761904733E-2</v>
       </c>
       <c r="N24" s="2">
         <v>6</v>
       </c>
       <c r="O24" s="2">
+        <v>6.032</v>
+      </c>
+      <c r="P24" s="2">
         <v>6.02</v>
-      </c>
-      <c r="P24" s="2">
-        <v>5.97</v>
       </c>
       <c r="Q24" s="2">
         <f t="shared" si="5"/>
-        <v>-1.9999999999999574E-2</v>
+        <v>-3.2000000000000028E-2</v>
       </c>
       <c r="R24" s="6">
         <f t="shared" si="6"/>
-        <v>67.633554817275751</v>
+        <v>68.064323607427056</v>
       </c>
       <c r="S24" s="6">
         <f t="shared" si="7"/>
-        <v>4.9999999999999822E-2</v>
-      </c>
-      <c r="T24" s="6">
-        <f>AVERAGE(S4:S24)</f>
-        <v>4.7368421052631574E-2</v>
+        <v>1.2000000000000455E-2</v>
+      </c>
+      <c r="T24" s="2" cm="1">
+        <f t="array" ref="T24">SUMPRODUCT(ABS(Q6:Q24))/COUNT(Q6:Q24)</f>
+        <v>1.7999999999999933E-2</v>
       </c>
     </row>
     <row r="31" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="S31" s="8" t="s">
-        <v>8</v>
-      </c>
+      <c r="S31" s="8"/>
     </row>
     <row r="49" spans="8:9" ht="15" x14ac:dyDescent="0.2">
       <c r="H49" s="7" t="s">
@@ -6154,10 +6181,10 @@
     </row>
     <row r="53" spans="8:9" ht="15" x14ac:dyDescent="0.2">
       <c r="H53" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="I53" s="7" t="s">
         <v>11</v>
-      </c>
-      <c r="I53" s="7" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="54" spans="8:9" x14ac:dyDescent="0.2">
@@ -6170,7 +6197,7 @@
     </row>
     <row r="55" spans="8:9" ht="15" x14ac:dyDescent="0.2">
       <c r="H55" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I55" s="2">
         <f>I54/H54</f>

</xml_diff>